<commit_message>
Stat of visual precention - model for
</commit_message>
<xml_diff>
--- a/Lingvistik_proj/ausen-emma_head_lingvistik.xlsx
+++ b/Lingvistik_proj/ausen-emma_head_lingvistik.xlsx
@@ -425,111 +425,116 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U43"/>
+  <dimension ref="A1:V43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Finding ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Tree sentences</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Found word</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Lemma</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Body category</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Language</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Name of work</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Before Nouns</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Before Adjektives</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Before Verbs</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Before Adverbs</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Before Pre- and postpositions</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Before Objects</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>After Nouns</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>After Adjektives</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>After Verbs</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>After Adverbs</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>After Pre- and postpositions</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>After Objects</t>
         </is>
@@ -538,94 +543,99 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>ausen-emma_S_2341_L_1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>"That is what you have in your head, I know and what you would certainly say if my father were not by."</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>"Especially when one of those two is such a fanciful, troublesome creature!" said Emma playfully. "That is what you have in your head, I know and what you would certainly say if my father were not by." "I believe it is very true, my dear, indeed," said Mr. Woodhouse, with a sigh.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>head, father</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>have, know, say</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>certainly</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>in, by</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ausen-emma_S_2727_L_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Emma turned away her head, divided between tears and smiles.</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>"But, Mr. Knightley, she is really very sorry to lose poor Miss Taylor, and I am sure she will miss her more than she thinks for." Emma turned away her head, divided between tears and smiles. "It is impossible that Emma should not miss such a companion," said Mr. Knightley.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>.</t>
@@ -633,74 +643,79 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>head, tears, smiles</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>turned, divided</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>away</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>between</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>ausen-emma_S_2936_L_3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Mr. Knightley shook his head at her.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>I made the match, you know, four years ago; and to have it take place, and be proved in the right, when so many people said Mr. Weston would never marry again, may comfort me for any thing." Mr. Knightley shook his head at her. Her father fondly replied, "Ah!</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>.</t>
@@ -708,70 +723,75 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>shook</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
         <is>
           <t>at</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>ausen-emma_S_11884_L_4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Mr. Elton was the very person fixed on by Emma for driving the young farmer out of Harriet's head.</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>She then repeated some warm personal praise which she had drawn from Mr. Elton, and now did full justice to; and Harriet blushed and smiled, and said she had always thought Mr. Elton very agreeable. Mr. Elton was the very person fixed on by Emma for driving the young farmer out of Harriet's head. She thought it would be an excellent match; and only too palpably desirable, natural, and probable, for her to have much merit in planning it.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>.</t>
@@ -779,74 +799,79 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>person, farmer, head</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>very, young</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>fixed, driving</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
         <is>
           <t>on, by, for, out, of</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>ausen-emma_S_13694_L_5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>There is health, not merely in her bloom, but in her air, her head, her glance.</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>what a bloom of full health, and such a pretty height and size; such a firm and upright figure! There is health, not merely in her bloom, but in her air, her head, her glance. One hears sometimes of a child being `the picture of health;' now, Emma always gives me the idea of being the complete picture of grown-up health.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>.</t>
@@ -854,74 +879,79 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>health, bloom, air, head, glance</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>is</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>merely</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>in, in</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>ausen-emma_S_16168_L_6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>He had nestled down his head most conveniently.</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>I took him as he was sleeping on the sofa, and it is as strong a likeness of his cockade as you would wish to see. He had nestled down his head most conveniently. That's very like.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>.</t>
@@ -929,74 +959,79 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>nestled</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>most, conveniently</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>down</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>ausen-emma_S_24059_L_7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Vanity working on a weak head, produces every sort of mischief.</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>You will puff her up with such ideas of her own beauty, and of what she has a claim to, that, in a little while, nobody within her reach will be good enough for her. Vanity working on a weak head, produces every sort of mischief. Nothing so easy as for a young lady to raise her expectations too high.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>.</t>
@@ -1004,74 +1039,79 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
           <t>Vanity, head, sort, mischief</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>weak</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>working, produces</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
         <is>
           <t>on, of</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>ausen-emma_S_26305_L_8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Miss Nash, head-teacher at Mrs. Goddard's, had written out at least three hundred; and Harriet, who had taken the first hint of it from her, hoped, with Miss Woodhouse's help, to get a great many more.</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>In this age of literature, such collections on a very grand scale are not uncommon. Miss Nash, head-teacher at Mrs. Goddard's, had written out at least three hundred; and Harriet, who had taken the first hint of it from her, hoped, with Miss Woodhouse's help, to get a great many more. Emma assisted with her invention, memory and taste; and as Harriet wrote a very pretty hand, it was likely to be an arrangement of the first order, in form as well as quantity.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>.</t>
@@ -1079,78 +1119,83 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>head, teacher, hint, help</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>first, great, many, more</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>written, taken, hoped, get</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>at, least</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>at, out, of, from, with</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ausen-emma_S_35885_L_9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>They had not been long seated and composed when Mr. Woodhouse, with a melancholy shake of the head and a sigh, called his daughter's attention to the sad change at Hartfield since she had been there last.</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>The beginning, however, of every visit displayed none but the properest feelings, and this being of necessity so short might be hoped to pass away in unsullied cordiality. They had not been long seated and composed when Mr. Woodhouse, with a melancholy shake of the head and a sigh, called his daughter's attention to the sad change at Hartfield since she had been there last. "Ah, my dear," said he, "poor Miss Taylor</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>.</t>
@@ -1158,78 +1203,83 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>shake, head, sigh, daughter, attention, change</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>melancholy, sad, last</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>seated, composed, called</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>long, there</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>with, of, to, at</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>ausen-emma_S_39630_L_10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>"I am sorry to hear you say so, sir; but I assure you, excepting those little nervous head-aches and palpitations which I am never entirely free from anywhere, I am quite well myself; and if the children were rather pale before they went to bed, it was only because they were a little more tired than usual, from their journey and the happiness of coming.</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Now I cannot say, that I think you are any of you looking well at present." "I am sorry to hear you say so, sir; but I assure you, excepting those little nervous head-aches and palpitations which I am never entirely free from anywhere, I am quite well myself; and if the children were rather pale before they went to bed, it was only because they were a little more tired than usual, from their journey and the happiness of coming. I hope you will think better of their looks to-morrow; for I assure you Mr. Wingfield told me, that he did not believe he had ever sent us off altogether, in such good case.</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>.</t>
@@ -1237,78 +1287,83 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
           <t>head, aches, palpitations, children, bed, journey, happiness</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>sorry, little, nervous, free, pale, tired, usual</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>hear, say, assure, excepting, went, coming</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>so, never, entirely, anywhere, quite, well, rather, only, little, more</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>from, to, than, from, of</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ausen-emma_S_40374_L_11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>"Ah!" said Mr. Woodhouse, shaking his head and fixing his eyes on her with tender concern.</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Here was a dangerous opening. "Ah!" said Mr. Woodhouse, shaking his head and fixing his eyes on her with tender concern. The ejaculation in Emma's ear expressed, "Ah! there is no end of the sad consequences of your going to South End.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>.</t>
@@ -1316,70 +1371,75 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>head, eyes, tender, concern</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr">
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
         <is>
           <t>said, shaking, fixing</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
         <is>
           <t>on, with</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>ausen-emma_S_41464_L_12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>How they were all to be conveyed, he would have made a difficulty if he could, but as his son and daughter's carriage and horses were actually at Hartfield, he was not able to make more than a simple question on that head; it hardly amounted to a doubt; nor did it occupy Emma long to convince him that they might in one of the carriages find room for Harriet also.</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Mr. Weston would take no denial; they must all dine at Randalls one day; even Mr. Woodhouse was persuaded to think it a possible thing in preference to a division of the party. How they were all to be conveyed, he would have made a difficulty if he could, but as his son and daughter's carriage and horses were actually at Hartfield, he was not able to make more than a simple question on that head; it hardly amounted to a doubt; nor did it occupy Emma long to convince him that they might in one of the carriages find room for Harriet also. Harriet, Mr. Elton, and Mr. Knightley, their own especial set, were the only persons invited to meet them; the hours were to be early, as well as the numbers few; Mr. Woodhouse's habits and inclination being consulted in every thing.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>.</t>
@@ -1387,78 +1447,83 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
           <t>difficulty, son, daughter, carriage, horses, question, head, doubt, carriages, room</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>able, more, simple</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>conveyed, made, make, amounted, occupy, convince, find</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>all, actually, hardly, long, also</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>at, than, on, to, in, of, for</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>ausen-emma_S_52610_L_13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>But he had fancied her in love with him; that evidently must have been his dependence; and after raving a little about the seeming incongruity of gentle manners and a conceited head, Emma was obliged in common honesty to stop and admit that her own behaviour to him had been so complaisant and obliging, so full of courtesy and attention, as (supposing her real motive unperceived) might warrant a man of ordinary observation and delicacy, like Mr. Elton, in fancying himself a very decided favourite.</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>The landed property of Hartfield certainly was inconsiderable, being but a sort of notch in the Donwell Abbey estate, to which all the rest of Highbury belonged; but their fortune, from other sources, was such as to make them scarcely secondary to Donwell Abbey itself, in every other kind of consequence; and the Woodhouses had long held a high place in the consideration of the neighbourhood which Mr. Elton had first entered not two years ago, to make his way as he could, without any alliances but in trade, or any thing to recommend him to notice but his situation and his civility. But he had fancied her in love with him; that evidently must have been his dependence; and after raving a little about the seeming incongruity of gentle manners and a conceited head, Emma was obliged in common honesty to stop and admit that her own behaviour to him had been so complaisant and obliging, so full of courtesy and attention, as (supposing her real motive unperceived) might warrant a man of ordinary observation and delicacy, like Mr. Elton, in fancying himself a very decided favourite. If she had so misinterpreted his feelings, she had little right to wonder that he , with self-interest to blind him, should have mistaken hers.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>.</t>
@@ -1466,157 +1531,167 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
           <t>love, dependence, incongruity, manners, head, honesty, behaviour, courtesy, attention, motive, man, observation, delicacy</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>little, gentle, conceited, common, own, complaisant, obliging, full, real, ordinary, favourite</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>fancied, raving, seeming, obliged, stop, admit, supposing, unperceived, warrant, fancying, decided</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>evidently, so, so, very</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>in, with, after, about, of, in, to, of, of, like, in</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>ausen-emma_S_68950_L_14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Harriet said, "very true," and she "would not think about it;" but still she talked of it still she could talk of nothing else; and Emma, at last, in order to put the Martins out of her head, was obliged to hurry on the news, which she had meant to give with so much tender caution; hardly knowing herself whether to rejoice or be angry, ashamed or only amused, at such a state of mind in poor Harriet such a conclusion of Mr. Elton's importance with her!</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>She exerted herself, and did try to make her comfortable, by considering all that had passed as a mere trifle, and quite unworthy of being dwelt on, "It might be distressing, for the moment," said she; "but you seem to have behaved extremely well; and it is over and may never can never, as a first meeting, occur again, and therefore you need not think about it." Harriet said, "very true," and she "would not think about it;" but still she talked of it still she could talk of nothing else; and Emma, at last, in order to put the Martins out of her head, was obliged to hurry on the news, which she had meant to give with so much tender caution; hardly knowing herself whether to rejoice or be angry, ashamed or only amused, at such a state of mind in poor Harriet such a conclusion of Mr. Elton's importance with her! Mr. Elton's rights, however, gradually revived.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
           <t>order, Martins, head, news, caution, state, mind, conclusion, importance</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>true, last, much, tender, angry, ashamed, poor</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>said, think, talked, talk, put, obliged, hurry, meant, give, knowing, rejoice, amused</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>very, still, still, else, so, hardly, only</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>about, of, of, at, in, out, of, on, with, at, of, in, of, with</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>ausen-emma_S_76580_L_15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>He shook his head and laughed.</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>At least you admire her except her complexion." He shook his head and laughed. "I cannot separate Miss Fairfax and her complexion."</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>.</t>
@@ -1624,41 +1699,45 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
         <is>
           <t>shook, laughed</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
@@ -1667,23 +1746,24 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>ausen-emma_S_83449_L_16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>"Yes, and what you told me on that head, confirmed an idea which I had entertained before.</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>We were speaking the other day, you know, of his being so warm an admirer of her performance." "Yes, and what you told me on that head, confirmed an idea which I had entertained before. I do not mean to reflect upon the good intentions of either Mr. Dixon or Miss Fairfax, but I cannot help suspecting either that, after making his proposals to her friend, he had the misfortune to fall in love with her , or that he became conscious of a little attachment on her side.</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>.</t>
@@ -1691,74 +1771,79 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
           <t>head, idea</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr">
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
         <is>
           <t>told, confirmed, entertained</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>before</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>on</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>ausen-emma_S_86346_L_17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>"Well," said Mrs. Weston, smiling, "you give him credit for more simple, disinterested benevolence in this instance than I do; for while Miss Bates was speaking, a suspicion darted into my head, and I have never been able to get it out again.</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>I know he had horses to-day for we arrived together; and I laughed at him about it, but he said not a word that could betray." "Well," said Mrs. Weston, smiling, "you give him credit for more simple, disinterested benevolence in this instance than I do; for while Miss Bates was speaking, a suspicion darted into my head, and I have never been able to get it out again. The more I think of it, the more probable it appears.</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>.</t>
@@ -1766,78 +1851,83 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>credit, benevolence, instance, suspicion, head</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>simple, disinterested, able</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>said, smiling, give, do, speaking, darted, get</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>more, never, again</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>for, in, for, into, out</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>ausen-emma_S_86843_L_18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Do not put it into his head.</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>I am sure he has not the least idea of it. Do not put it into his head. Why should he marry?</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>.</t>
@@ -1845,70 +1935,75 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
         <is>
           <t>put</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
         <is>
           <t>into</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>ausen-emma_S_93472_L_19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>He shook his head with a smile, and looked as if he had very little doubt and very little mercy.</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Do not distress her." He shook his head with a smile, and looked as if he had very little doubt and very little mercy. Soon afterwards he began again, "How much your friends in Ireland must be enjoying your pleasure on this occasion, Miss Fairfax.</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>.</t>
@@ -1916,78 +2011,83 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>head, smile, doubt, mercy</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>little, little</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>shook, looked, had</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="N20" t="inlineStr">
         <is>
           <t>very, very</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>with</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>ausen-emma_S_94613_L_20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>But Emma still shook her head in steady scepticism.</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>The listeners were amused; and Mrs. Weston gave Emma a look of particular meaning. But Emma still shook her head in steady scepticism. "So obliged to you!</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>.</t>
@@ -1995,153 +2095,163 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
           <t>head, scepticism</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>steady</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>shook</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>still</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>ausen-emma_S_100395_L_21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>"Ah! (shaking his head) the uncertainty of when I may be able to return!</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>"This will not be your only visit to Randalls." "Ah! (shaking his head) the uncertainty of when I may be able to return! I shall try for it with a zeal!</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
           <t>head, uncertainty</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>able</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>shaking, return</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
         <is>
           <t>of</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>ausen-emma_S_102584_L_22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>When his letter to Mrs. Weston arrived, Emma had the perusal of it; and she read it with a degree of pleasure and admiration which made her at first shake her head over her own sensations, and think she had undervalued their strength.</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>I shall do very well again after a little while and then, it will be a good thing over; for they say every body is in love once in their lives, and I shall have been let off easily." When his letter to Mrs. Weston arrived, Emma had the perusal of it; and she read it with a degree of pleasure and admiration which made her at first shake her head over her own sensations, and think she had undervalued their strength. It was a long, well-written letter, giving the particulars of his journey and of his feelings, expressing all the affection, gratitude, and respect which was natural and honourable, and describing every thing exterior and local that could be supposed attractive, with spirit and precision.</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>.</t>
@@ -2149,78 +2259,83 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
           <t>letter, perusal, degree, pleasure, admiration, head, sensations, strength</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>own</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>arrived, had, read, made, shake, think, undervalued</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>first</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>to, of, with, of, at, over</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr"/>
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>ausen-emma_S_104031_L_23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>Warmth and tenderness of heart, with an affectionate, open manner, will beat all the clearness of head in the world, for attraction, I am sure it will.</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>"There is nothing to be compared to it. Warmth and tenderness of heart, with an affectionate, open manner, will beat all the clearness of head in the world, for attraction, I am sure it will. It is tenderness of heart which makes my dear father so generally beloved which gives Isabella all her popularity.</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>.</t>
@@ -2228,74 +2343,79 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>Warmth, tenderness, heart, manner, clearness, head, world, attraction</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>affectionate, open, sure</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>beat</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
         <is>
           <t>of, with, of, in, for</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>ausen-emma_S_104106_L_24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>I would not change you for the clearest-headed, longest-sighted, best-judging female breathing.</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Dear Harriet! I would not change you for the clearest-headed, longest-sighted, best-judging female breathing. Oh!</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>.</t>
@@ -2303,78 +2423,83 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
           <t>breathing</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>longest, female</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>change, headed, sighted, judging</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>clearest, best</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>for</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>ausen-emma_S_107310_L_25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>"No, indeed, I have no doubts at all on that head.</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>"We cannot suppose," said Emma, smiling, "that Mr. Elton would hesitate to assure you of there being a very musical society in Highbury; and I hope you will not find he has outstepped the truth more than may be pardoned, in consideration of the motive." "No, indeed, I have no doubts at all on that head. I am delighted to find myself in such a circle.</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>.</t>
@@ -2382,74 +2507,79 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
           <t>doubts, head</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr">
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
         <is>
           <t>have</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>indeed, at, all</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>on</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>ausen-emma_S_112173_L_26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>No till Cole alluded to my supposed attachment, it had never entered my head.</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>She is reserved, more reserved, I think, than she used to be And I love an open temper. No till Cole alluded to my supposed attachment, it had never entered my head. I saw Jane Fairfax and conversed with her, with admiration and pleasure always but with no thought beyond."</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>.</t>
@@ -2457,149 +2587,159 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
           <t>attachment, head</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr">
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
         <is>
           <t>alluded, supposed, entered</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>never</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>to</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>ausen-emma_S_116281_L_27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>"I not aware!" said Jane, shaking her head; "dear Mrs. Elton, who can have thought of it as I have done?"</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>my dear, we cannot begin too early; you are not aware of the difficulty of procuring exactly the desirable thing." "I not aware!" said Jane, shaking her head; "dear Mrs. Elton, who can have thought of it as I have done?" "But you have not seen so much of the world as I have.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>austen-emma.txt</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
           <t>aware, dear</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>said, shaking, thought, done</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
         <is>
           <t>of</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
       <c r="Q28" t="inlineStr"/>
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>ausen-emma_S_119658_L_28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>"She has taken it into her head that Enscombe is too cold for her.</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>To Bath, or to Clifton?" "She has taken it into her head that Enscombe is too cold for her. The fact is, I suppose, that she is tired of Enscombe.</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>.</t>
@@ -2607,78 +2747,83 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>austen-emma.txt</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
           <t>cold</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>taken</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>too</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>into, for</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>ausen-emma_S_126934_L_29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>She was not yet dancing; she was working her way up from the bottom, and had therefore leisure to look around, and by only turning her head a little she saw it all.</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Emma saw it. She was not yet dancing; she was working her way up from the bottom, and had therefore leisure to look around, and by only turning her head a little she saw it all. When she was half-way up the set, the whole group were exactly behind her, and she would no longer allow her eyes to watch; but Mr. Elton was so near, that she heard every syllable of a dialogue which just then took place between him and Mrs. Weston; and she perceived that his wife, who was standing immediately above her, was not only listening also, but even encouraging him by significant glances.</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>.</t>
@@ -2686,78 +2831,83 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
           <t>way, bottom, leisure, head</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>dancing, working, had, look, turning, saw</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>yet, up, therefore, around, only</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>from, by</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr"/>
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>ausen-emma_S_128454_L_30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>He shook his head; but there was a smile of indulgence with it, and he only said, "I shall not scold you.</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>"I did," replied Emma, "and they cannot forgive me." He shook his head; but there was a smile of indulgence with it, and he only said, "I shall not scold you. I leave you to your own reflections."</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>.</t>
@@ -2765,74 +2915,79 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
           <t>head, smile, indulgence</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr">
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
         <is>
           <t>shook, was, said, scold</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>only</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>of, with</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>ausen-emma_S_129603_L_31</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>How the trampers might have behaved, had the young ladies been more courageous, must be doubtful; but such an invitation for attack could not be resisted; and Harriet was soon assailed by half a dozen children, headed by a stout woman and a great boy, all clamorous, and impertinent in look, though not absolutely in word.</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>She had suffered very much from cramp after dancing, and her first attempt to mount the bank brought on such a return of it as made her absolutely powerless and in this state, and exceedingly terrified, she had been obliged to remain. How the trampers might have behaved, had the young ladies been more courageous, must be doubtful; but such an invitation for attack could not be resisted; and Harriet was soon assailed by half a dozen children, headed by a stout woman and a great boy, all clamorous, and impertinent in look, though not absolutely in word. More and more frightened, she immediately promised them money, and taking out her purse, gave them a shilling, and begged them not to want more, or to use her ill.</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>.</t>
@@ -2840,153 +2995,163 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
           <t>trampers, ladies, invitation, attack, dozen, children, woman, boy, look, word</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>young, courageous, doubtful, stout, great, clamorous</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>behaved, had, resisted, assailed, headed, impertinent</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>more, soon, all, absolutely</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>for, by, by, in, in</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>ausen-emma_S_136556_L_32</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>And how could it possibly come into your head?"</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>she cried with a most open eagerness "Never, for the twentieth part of a moment, did such an idea occur to me. And how could it possibly come into your head?" "I have lately imagined that I saw symptoms of attachment between them certain expressive looks, which I did not believe meant to be public."</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
         <is>
           <t>come</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>possibly</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>into</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr"/>
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>ausen-emma_S_149874_L_33</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>And poor John's son came to talk to Mr. Elton about relief from the parish; he is very well to do himself, you know, being head man at the Crown, ostler, and every thing of that sort, but still he cannot keep his father without some help; and so, when Mr. Elton came back, he told us what John ostler had been telling him, and then it came out about the chaise having been sent to Randalls to take Mr. Frank Churchill to Richmond.</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Poor old John, I have a great regard for him; he was clerk to my poor father twenty-seven years; and now, poor old man, he is bed-ridden, and very poorly with the rheumatic gout in his joints I must go and see him to-day; and so will Jane, I am sure, if she gets out at all. And poor John's son came to talk to Mr. Elton about relief from the parish; he is very well to do himself, you know, being head man at the Crown, ostler, and every thing of that sort, but still he cannot keep his father without some help; and so, when Mr. Elton came back, he told us what John ostler had been telling him, and then it came out about the chaise having been sent to Randalls to take Mr. Frank Churchill to Richmond. That was what happened before tea.</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>.</t>
@@ -2994,78 +3159,83 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
           <t>son, relief, head, man, ostler, thing, sort, father, help, ostler, chaise</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>poor, well</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>came, talk, do, know, keep, came, told, telling, came, sent, take</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>very, still, so, back, then</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>to, about, from, at, of, without, out, about, to, to</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>ausen-emma_S_150755_L_34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>Emma's colour was heightened by this unjust praise; and with a smile, and shake of the head, which spoke much, she looked at Mr. Knightley.</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>She is always so attentive to them!" Emma's colour was heightened by this unjust praise; and with a smile, and shake of the head, which spoke much, she looked at Mr. Knightley. It seemed as if there were an instantaneous impression in her favour, as if his eyes received the truth from her's, and all that had passed of good in her feelings were at once caught and honoured.</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>.</t>
@@ -3073,78 +3243,83 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
           <t>colour, praise, smile, shake, head</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>unjust</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>heightened, spoke, looked</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>much</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>by, with, of, at</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>ausen-emma_S_151760_L_35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Even Mr. Weston shook his head, and looked solemn, and said, "Ah! poor woman, who would have thought it!" and resolved, that his mourning should be as handsome as possible; and his wife sat sighing and moralising over her broad hems with a commiseration and good sense, true and steady.</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Mr. Churchill would never get over it." Even Mr. Weston shook his head, and looked solemn, and said, "Ah! poor woman, who would have thought it!" and resolved, that his mourning should be as handsome as possible; and his wife sat sighing and moralising over her broad hems with a commiseration and good sense, true and steady. How it would affect Frank was among the earliest thoughts of both.</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>.</t>
@@ -3152,78 +3327,83 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
           <t>head, woman, mourning, wife, hems, commiseration, sense</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>solemn, !, poor, handsome, possible, broad, good, true, steady</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>shook, looked, said, thought, resolved, sat, sighing, moralising</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="N36" t="inlineStr">
         <is>
           <t>Even, as</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>as, over, with</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>ausen-emma_S_156585_L_36</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>"I am quite easy on that head," replied Mrs. Weston.</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>They must take the consequence, if they have heard each other spoken of in a way not perfectly agreeable!" "I am quite easy on that head," replied Mrs. Weston. "I am very sure that I never said any thing of either to the other, which both might not have heard."</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>.</t>
@@ -3231,149 +3411,159 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>austen-emma.txt</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>replied</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>quite</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>on</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>ausen-emma_S_161276_L_37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>The blunders, the blindness of her own head and heart!</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>How to understand the deceptions she had been thus practising on herself, and living under! The blunders, the blindness of her own head and heart! she sat still, she walked about, she tried her own room, she tried the shrubbery in every place, every posture, she perceived that she had acted most weakly; that she had been imposed on by others in a most mortifying degree; that she had been imposing on herself in a degree yet more mortifying; that she was wretched, and should probably find this day but the beginning of wretchedness.</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>head</t>
-        </is>
-      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
           <t>blunders, blindness, head, heart</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>own</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
         <is>
           <t>of</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>ausen-emma_S_174778_L_38</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>When he came to Miss Woodhouse, he was obliged to read the whole of it aloud all that related to her, with a smile; a look; a shake of the head; a word or two of assent, or disapprobation; or merely of love, as the subject required; concluding, however, seriously, and, after steady reflection, thus "Very bad though it might have been worse.</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>"I was not quite impartial in my judgment, Emma: but yet, I think had you not been in the case I should still have distrusted him." When he came to Miss Woodhouse, he was obliged to read the whole of it aloud all that related to her, with a smile; a look; a shake of the head; a word or two of assent, or disapprobation; or merely of love, as the subject required; concluding, however, seriously, and, after steady reflection, thus "Very bad though it might have been worse. Playing a most dangerous game.</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>.</t>
@@ -3381,78 +3571,83 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
           <t>whole, smile, look, shake, head, word, assent, disapprobation, love, subject, reflection</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>steady, bad, worse</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>came, obliged, read, related, required, concluding</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>aloud, merely, however, seriously, thus, Very</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>to, of, to, with, of, of, of, after</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>ausen-emma_S_178199_L_39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>And again, on Emma's merely turning her head to look at Mrs. Bates's knitting, she added, in a half whisper, "I mentioned no names , you will observe.</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>My representation, you see, has quite appeased her." And again, on Emma's merely turning her head to look at Mrs. Bates's knitting, she added, in a half whisper, "I mentioned no names , you will observe. Oh!</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>.</t>
@@ -3460,74 +3655,79 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
           <t>head, knitting, half, whisper, names</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr">
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
         <is>
           <t>turning, look, added, mentioned, observe</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>again, merely</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>on, at, in</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>ausen-emma_S_186688_L_40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>"Me!" cried Emma, shaking her head.</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Much of this, I have no doubt, she may thank you for." "Me!" cried Emma, shaking her head. "Ah! poor Harriet!"</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>.</t>
@@ -3535,41 +3735,45 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>head</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr">
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>head</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
         <is>
           <t>cried, shaking</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr"/>
@@ -3578,23 +3782,24 @@
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>ausen-emma_S_188417_L_41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>You will be glad to hear (inclining his head, and whispering seriously) that my uncle means to give her all my aunt's jewels.</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Observe her eyes, as she is looking up at my father. You will be glad to hear (inclining his head, and whispering seriously) that my uncle means to give her all my aunt's jewels. They are to be new set.</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>.</t>
@@ -3602,50 +3807,54 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
           <t>head, uncle, aunt, jewels</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>glad</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>hear, inclining, whispering, means, give</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>seriously</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
@@ -3653,23 +3862,24 @@
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>ausen-emma_S_188454_L_42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>I am resolved to have some in an ornament for the head.</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>They are to be new set. I am resolved to have some in an ornament for the head. Will not it be beautiful in her dark hair?"</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>.</t>
@@ -3677,53 +3887,58 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>head</t>
+          <t>.</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>body part</t>
+          <t>head</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>body part</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>NLTK Gutenberg</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>austen-emma.txt</t>
+          <t>NLTK Gutenberg</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
+          <t>austen-emma.txt</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
           <t>ornament, head</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr">
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
         <is>
           <t>resolved, have</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr">
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
         <is>
           <t>in, for</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>